<commit_message>
Add combat data updates and PlayMode smoke coverage
</commit_message>
<xml_diff>
--- a/JsonFile/Assets/ExcelFiles/Patch_Note.xlsx
+++ b/JsonFile/Assets/ExcelFiles/Patch_Note.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Adventure\JsonFile\Assets\ExcelFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\OneDrive\문서\Unity\Adventure\JsonFile\Assets\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{007728E5-DAAA-4C46-8F8E-BBC59C9C71D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D779F4B9-72AE-4E88-A74F-19C2DB85677C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Patch_Notes" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>version</t>
   </si>
@@ -62,6 +62,14 @@
     <t>["텍스트 출력 부분 버그 수정",
 "이벤트에서 지 마음대로 버튼 생성 되는 경우 수정 ",
 "텍스트에 웨이브 기능 예외처리 추가"]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.0.4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>["TC테스트용 추가 패치노트"]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -449,8 +457,15 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="2">
+        <v>46185</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B6" s="2"/>

</xml_diff>